<commit_message>
feat: tich hop 4 video thuc chien Don Nu tu D:\Code_Tino_01_09\Video\Video_don nu
</commit_message>
<xml_diff>
--- a/Gioi_Thieu_Tinh_Nang_Badminton_Pro.xlsx
+++ b/Gioi_Thieu_Tinh_Nang_Badminton_Pro.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="408" uniqueCount="346">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="432" uniqueCount="367">
   <si>
     <t>BÁO CÁO TỔNG QUAN HỆ THỐNG BADMINTON PRO TRAINER</t>
   </si>
@@ -81,10 +81,10 @@
     <t>Hình ảnh mô phỏng trực quan</t>
   </si>
   <si>
-    <t>9 VIDEO THỰC TẾ ĐƠN NAM &amp; ĐÔI NAM</t>
-  </si>
-  <si>
-    <t>6 Bài Đơn Nam + 3 Bài Đôi Nam, chống tua, tự động đổi theo ô sân</t>
+    <t>13 VIDEO THỰC TẾ (ĐƠN NAM, ĐÔI NAM, ĐƠN NỮ)</t>
+  </si>
+  <si>
+    <t>6 Đơn Nam + 3 Đôi Nam + 4 Đơn Nữ, chống tua, tự động đổi theo ô sân</t>
   </si>
   <si>
     <t>100% Video thực tế</t>
@@ -720,7 +720,7 @@
     <t>Bắt đối thủ phải lao hết tốc lực cứu cầu lưới</t>
   </si>
   <si>
-    <t>DANH MỤC 9 VIDEO THỰC CHIẾN &amp; CÔNG NGHỆ GẮN LINK VIDEO</t>
+    <t>DANH MỤC 13 VIDEO THỰC CHIẾN (ĐƠN NAM, ĐÔI NAM, ĐƠN NỮ) &amp; CÔNG NGHỆ GẮN LINK</t>
   </si>
   <si>
     <t>CHUYÊN MỤC</t>
@@ -880,6 +880,69 @@
   </si>
   <si>
     <t>10</t>
+  </si>
+  <si>
+    <t>ĐƠN NỮ</t>
+  </si>
+  <si>
+    <t>Kỹ Thuật Di Chuyển Bộ Pháp Dẻo Dai &amp; Điều Cầu Đơn Nữ</t>
+  </si>
+  <si>
+    <t>Bộ pháp linh hoạt, di chuyển 4 góc sân êm ái và hồi vị nhịp nhàng.</t>
+  </si>
+  <si>
+    <t>snaptik.vn_7500378802141269256.mp4</t>
+  </si>
+  <si>
+    <t>Chống tua nhanh, tự động tích xanh, xem chậm 0.5x</t>
+  </si>
+  <si>
+    <t>11</t>
+  </si>
+  <si>
+    <t>Chiến Thuật Ép Cầu Đáy Sân &amp; Mở Góc Tấn Công Đơn Nữ</t>
+  </si>
+  <si>
+    <t>Kỹ thuật phông cầu cao sâu, khai thác khoảng trống hai góc biên.</t>
+  </si>
+  <si>
+    <t>snaptik.vn_7567643845215669521.mp4</t>
+  </si>
+  <si>
+    <t>Chống tua nhanh, tự động tích xanh, xem toàn màn hình</t>
+  </si>
+  <si>
+    <t>12</t>
+  </si>
+  <si>
+    <t>Kỹ Thuật Bỏ Nhỏ Sát Lưới &amp; Kéo Lưới Lừa Hướng Đơn Nữ</t>
+  </si>
+  <si>
+    <t>Cảm giác mặt vợt tinh tế, cắt cầu đổi hướng đánh gục phản xạ.</t>
+  </si>
+  <si>
+    <t>snaptik.vn_7598797082912181511.mp4</t>
+  </si>
+  <si>
+    <t>Chống tua nhanh, tự động tích xanh, quay chậm</t>
+  </si>
+  <si>
+    <t>13</t>
+  </si>
+  <si>
+    <t>Kỹ Năng Đập Cầu Điểm Rơi &amp; Chém Cầu Bạt Góc Đơn Nữ</t>
+  </si>
+  <si>
+    <t>Biến hóa giữa đập cắm biên và chém cầu rơi chéo sân dứt điểm.</t>
+  </si>
+  <si>
+    <t>snaptik.vn_7651286512998288661.mp4</t>
+  </si>
+  <si>
+    <t>Chống tua nhanh, tự động tích xanh, âm thanh chuẩn</t>
+  </si>
+  <si>
+    <t>14</t>
   </si>
   <si>
     <t>TÍNH NĂNG MỞ RỘNG</t>
@@ -2820,7 +2883,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -3059,6 +3122,86 @@
       </c>
       <c r="F12" s="28" t="s">
         <v>292</v>
+      </c>
+    </row>
+    <row r="13" ht="36" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" s="23" t="s">
+        <v>293</v>
+      </c>
+      <c r="B13" s="24" t="s">
+        <v>288</v>
+      </c>
+      <c r="C13" s="25" t="s">
+        <v>294</v>
+      </c>
+      <c r="D13" s="25" t="s">
+        <v>295</v>
+      </c>
+      <c r="E13" s="25" t="s">
+        <v>296</v>
+      </c>
+      <c r="F13" s="25" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="14" ht="36" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" s="26" t="s">
+        <v>298</v>
+      </c>
+      <c r="B14" s="27" t="s">
+        <v>288</v>
+      </c>
+      <c r="C14" s="28" t="s">
+        <v>299</v>
+      </c>
+      <c r="D14" s="28" t="s">
+        <v>300</v>
+      </c>
+      <c r="E14" s="28" t="s">
+        <v>301</v>
+      </c>
+      <c r="F14" s="28" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="15" ht="36" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" s="23" t="s">
+        <v>303</v>
+      </c>
+      <c r="B15" s="24" t="s">
+        <v>288</v>
+      </c>
+      <c r="C15" s="25" t="s">
+        <v>304</v>
+      </c>
+      <c r="D15" s="25" t="s">
+        <v>305</v>
+      </c>
+      <c r="E15" s="25" t="s">
+        <v>306</v>
+      </c>
+      <c r="F15" s="25" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="16" ht="36" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" s="26" t="s">
+        <v>308</v>
+      </c>
+      <c r="B16" s="27" t="s">
+        <v>309</v>
+      </c>
+      <c r="C16" s="28" t="s">
+        <v>310</v>
+      </c>
+      <c r="D16" s="28" t="s">
+        <v>311</v>
+      </c>
+      <c r="E16" s="28" t="s">
+        <v>312</v>
+      </c>
+      <c r="F16" s="28" t="s">
+        <v>313</v>
       </c>
     </row>
   </sheetData>
@@ -3084,7 +3227,7 @@
   <sheetData>
     <row r="1" ht="36" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="39" t="s">
-        <v>293</v>
+        <v>314</v>
       </c>
       <c r="B1" s="39"/>
       <c r="C1" s="39"/>
@@ -3093,104 +3236,104 @@
     </row>
     <row r="2" ht="28" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="40" t="s">
-        <v>294</v>
+        <v>315</v>
       </c>
       <c r="B2" s="40" t="s">
-        <v>295</v>
+        <v>316</v>
       </c>
       <c r="C2" s="40" t="s">
-        <v>296</v>
+        <v>317</v>
       </c>
       <c r="D2" s="40" t="s">
-        <v>297</v>
+        <v>318</v>
       </c>
       <c r="E2" s="40" t="s">
-        <v>298</v>
+        <v>319</v>
       </c>
     </row>
     <row r="3" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="23" t="s">
-        <v>299</v>
+        <v>320</v>
       </c>
       <c r="B3" s="23" t="s">
-        <v>300</v>
+        <v>321</v>
       </c>
       <c r="C3" s="24" t="s">
-        <v>301</v>
+        <v>322</v>
       </c>
       <c r="D3" s="25" t="s">
-        <v>302</v>
+        <v>323</v>
       </c>
       <c r="E3" s="25" t="s">
-        <v>303</v>
+        <v>324</v>
       </c>
     </row>
     <row r="4" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="26" t="s">
-        <v>304</v>
+        <v>325</v>
       </c>
       <c r="B4" s="26" t="s">
-        <v>305</v>
+        <v>326</v>
       </c>
       <c r="C4" s="27" t="s">
-        <v>306</v>
+        <v>327</v>
       </c>
       <c r="D4" s="28" t="s">
-        <v>307</v>
+        <v>328</v>
       </c>
       <c r="E4" s="28" t="s">
-        <v>308</v>
+        <v>329</v>
       </c>
     </row>
     <row r="5" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="23" t="s">
-        <v>309</v>
+        <v>330</v>
       </c>
       <c r="B5" s="23" t="s">
-        <v>310</v>
+        <v>331</v>
       </c>
       <c r="C5" s="24" t="s">
-        <v>311</v>
+        <v>332</v>
       </c>
       <c r="D5" s="25" t="s">
-        <v>312</v>
+        <v>333</v>
       </c>
       <c r="E5" s="25" t="s">
-        <v>313</v>
+        <v>334</v>
       </c>
     </row>
     <row r="6" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="26" t="s">
-        <v>314</v>
+        <v>335</v>
       </c>
       <c r="B6" s="26" t="s">
-        <v>315</v>
+        <v>336</v>
       </c>
       <c r="C6" s="27" t="s">
-        <v>316</v>
+        <v>337</v>
       </c>
       <c r="D6" s="28" t="s">
-        <v>317</v>
+        <v>338</v>
       </c>
       <c r="E6" s="28" t="s">
-        <v>318</v>
+        <v>339</v>
       </c>
     </row>
     <row r="7" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="23" t="s">
-        <v>319</v>
+        <v>340</v>
       </c>
       <c r="B7" s="23" t="s">
-        <v>320</v>
+        <v>341</v>
       </c>
       <c r="C7" s="24" t="s">
-        <v>321</v>
+        <v>342</v>
       </c>
       <c r="D7" s="25" t="s">
-        <v>322</v>
+        <v>343</v>
       </c>
       <c r="E7" s="25" t="s">
-        <v>323</v>
+        <v>344</v>
       </c>
     </row>
   </sheetData>
@@ -3214,86 +3357,86 @@
   <sheetData>
     <row r="1" ht="36" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="41" t="s">
-        <v>324</v>
+        <v>345</v>
       </c>
       <c r="B1" s="41"/>
       <c r="C1" s="41"/>
     </row>
     <row r="2" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="42" t="s">
-        <v>325</v>
+        <v>346</v>
       </c>
       <c r="B2" s="42" t="s">
-        <v>326</v>
+        <v>347</v>
       </c>
       <c r="C2" s="42" t="s">
-        <v>327</v>
+        <v>348</v>
       </c>
     </row>
     <row r="3" ht="42" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="15" t="s">
-        <v>328</v>
+        <v>349</v>
       </c>
       <c r="B3" s="16" t="s">
-        <v>329</v>
+        <v>350</v>
       </c>
       <c r="C3" s="17" t="s">
-        <v>330</v>
+        <v>351</v>
       </c>
     </row>
     <row r="4" ht="42" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="18" t="s">
-        <v>331</v>
+        <v>352</v>
       </c>
       <c r="B4" s="19" t="s">
-        <v>332</v>
+        <v>353</v>
       </c>
       <c r="C4" s="20" t="s">
-        <v>333</v>
+        <v>354</v>
       </c>
     </row>
     <row r="5" ht="42" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="15" t="s">
-        <v>334</v>
+        <v>355</v>
       </c>
       <c r="B5" s="16" t="s">
-        <v>335</v>
+        <v>356</v>
       </c>
       <c r="C5" s="17" t="s">
-        <v>336</v>
+        <v>357</v>
       </c>
     </row>
     <row r="6" ht="42" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="18" t="s">
-        <v>337</v>
+        <v>358</v>
       </c>
       <c r="B6" s="19" t="s">
-        <v>338</v>
+        <v>359</v>
       </c>
       <c r="C6" s="20" t="s">
-        <v>339</v>
+        <v>360</v>
       </c>
     </row>
     <row r="7" ht="42" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="15" t="s">
-        <v>340</v>
+        <v>361</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>341</v>
+        <v>362</v>
       </c>
       <c r="C7" s="17" t="s">
-        <v>342</v>
+        <v>363</v>
       </c>
     </row>
     <row r="8" ht="42" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="18" t="s">
-        <v>343</v>
+        <v>364</v>
       </c>
       <c r="B8" s="19" t="s">
-        <v>344</v>
+        <v>365</v>
       </c>
       <c r="C8" s="20" t="s">
-        <v>345</v>
+        <v>366</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: tich hop 4 video thuc chien Doi Nu tu D:\Code_Tino_01_09\Video\Video_doi nu
</commit_message>
<xml_diff>
--- a/Gioi_Thieu_Tinh_Nang_Badminton_Pro.xlsx
+++ b/Gioi_Thieu_Tinh_Nang_Badminton_Pro.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="432" uniqueCount="367">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="456" uniqueCount="386">
   <si>
     <t>BÁO CÁO TỔNG QUAN HỆ THỐNG BADMINTON PRO TRAINER</t>
   </si>
@@ -81,10 +81,10 @@
     <t>Hình ảnh mô phỏng trực quan</t>
   </si>
   <si>
-    <t>13 VIDEO THỰC TẾ (ĐƠN NAM, ĐÔI NAM, ĐƠN NỮ)</t>
-  </si>
-  <si>
-    <t>6 Đơn Nam + 3 Đôi Nam + 4 Đơn Nữ, chống tua, tự động đổi theo ô sân</t>
+    <t>17 VIDEO THỰC TẾ (4 CHUYÊN MỤC)</t>
+  </si>
+  <si>
+    <t>6 Đơn Nam + 3 Đôi Nam + 4 Đơn Nữ + 4 Đôi Nữ, chống tua, tự động đổi theo ô sân</t>
   </si>
   <si>
     <t>100% Video thực tế</t>
@@ -720,7 +720,7 @@
     <t>Bắt đối thủ phải lao hết tốc lực cứu cầu lưới</t>
   </si>
   <si>
-    <t>DANH MỤC 13 VIDEO THỰC CHIẾN (ĐƠN NAM, ĐÔI NAM, ĐƠN NỮ) &amp; CÔNG NGHỆ GẮN LINK</t>
+    <t>DANH MỤC 17 VIDEO THỰC CHIẾN (ĐƠN NAM, ĐÔI NAM, ĐƠN NỮ, ĐÔI NỮ) &amp; CÔNG NGHỆ GẮN LINK</t>
   </si>
   <si>
     <t>CHUYÊN MỤC</t>
@@ -943,6 +943,63 @@
   </si>
   <si>
     <t>14</t>
+  </si>
+  <si>
+    <t>ĐÔI NỮ</t>
+  </si>
+  <si>
+    <t>Chiến Thuật Bọc Lót &amp; Phòng Thủ Bền Bỉ Đôi Nữ</t>
+  </si>
+  <si>
+    <t>Phối hợp di chuyển bọc lót, cứu cầu liên hoàn và phá thế tấn công.</t>
+  </si>
+  <si>
+    <t>snaptik.vn_7372888645730192658.mp4</t>
+  </si>
+  <si>
+    <t>15</t>
+  </si>
+  <si>
+    <t>Kỹ Thuật Phản Tạt Đè Cầu &amp; Gài Lưới Đôi Nữ</t>
+  </si>
+  <si>
+    <t>Giữ thế chủ động trên lưới, tạt cầu thấp không cho đối thủ nâng bổng.</t>
+  </si>
+  <si>
+    <t>snaptik.vn_7495761376141397255.mp4</t>
+  </si>
+  <si>
+    <t>16</t>
+  </si>
+  <si>
+    <t>Đổi Vị Trí Công - Thủ &amp; Chuyển Giao Quyền Tấn Công</t>
+  </si>
+  <si>
+    <t>Quy tắc di chuyển hoán đổi trước - sau trong trận đấu đôi nữ.</t>
+  </si>
+  <si>
+    <t>snaptik.vn_7669811035297172757.mp4</t>
+  </si>
+  <si>
+    <t>Chống tua nhanh, tự động tích xanh, tua lại 5s</t>
+  </si>
+  <si>
+    <t>17</t>
+  </si>
+  <si>
+    <t>Tấn Công Liên Hoàn Đập Cầu &amp; Bắt Lưới Dứt Điểm Đôi Nữ</t>
+  </si>
+  <si>
+    <t>Phối hợp nhịp nhàng giữa quả đập phía sau và quả chớp lưới phía trước.</t>
+  </si>
+  <si>
+    <t>snaptik.vn_7681640086798159124.mp4</t>
+  </si>
+  <si>
+    <t>Chống tua nhanh, tự động tích xanh, âm thanh sống động</t>
+  </si>
+  <si>
+    <t>18</t>
   </si>
   <si>
     <t>TÍNH NĂNG MỞ RỘNG</t>
@@ -2883,7 +2940,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F20"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -3201,7 +3258,87 @@
         <v>312</v>
       </c>
       <c r="F16" s="28" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="17" ht="36" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" s="23" t="s">
         <v>313</v>
+      </c>
+      <c r="B17" s="24" t="s">
+        <v>309</v>
+      </c>
+      <c r="C17" s="25" t="s">
+        <v>314</v>
+      </c>
+      <c r="D17" s="25" t="s">
+        <v>315</v>
+      </c>
+      <c r="E17" s="25" t="s">
+        <v>316</v>
+      </c>
+      <c r="F17" s="25" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="18" ht="36" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" s="26" t="s">
+        <v>317</v>
+      </c>
+      <c r="B18" s="27" t="s">
+        <v>309</v>
+      </c>
+      <c r="C18" s="28" t="s">
+        <v>318</v>
+      </c>
+      <c r="D18" s="28" t="s">
+        <v>319</v>
+      </c>
+      <c r="E18" s="28" t="s">
+        <v>320</v>
+      </c>
+      <c r="F18" s="28" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="19" ht="36" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" s="23" t="s">
+        <v>322</v>
+      </c>
+      <c r="B19" s="24" t="s">
+        <v>309</v>
+      </c>
+      <c r="C19" s="25" t="s">
+        <v>323</v>
+      </c>
+      <c r="D19" s="25" t="s">
+        <v>324</v>
+      </c>
+      <c r="E19" s="25" t="s">
+        <v>325</v>
+      </c>
+      <c r="F19" s="25" t="s">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="20" ht="36" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" s="26" t="s">
+        <v>327</v>
+      </c>
+      <c r="B20" s="27" t="s">
+        <v>328</v>
+      </c>
+      <c r="C20" s="28" t="s">
+        <v>329</v>
+      </c>
+      <c r="D20" s="28" t="s">
+        <v>330</v>
+      </c>
+      <c r="E20" s="28" t="s">
+        <v>331</v>
+      </c>
+      <c r="F20" s="28" t="s">
+        <v>332</v>
       </c>
     </row>
   </sheetData>
@@ -3227,7 +3364,7 @@
   <sheetData>
     <row r="1" ht="36" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="39" t="s">
-        <v>314</v>
+        <v>333</v>
       </c>
       <c r="B1" s="39"/>
       <c r="C1" s="39"/>
@@ -3236,104 +3373,104 @@
     </row>
     <row r="2" ht="28" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="40" t="s">
-        <v>315</v>
+        <v>334</v>
       </c>
       <c r="B2" s="40" t="s">
-        <v>316</v>
+        <v>335</v>
       </c>
       <c r="C2" s="40" t="s">
-        <v>317</v>
+        <v>336</v>
       </c>
       <c r="D2" s="40" t="s">
-        <v>318</v>
+        <v>337</v>
       </c>
       <c r="E2" s="40" t="s">
-        <v>319</v>
+        <v>338</v>
       </c>
     </row>
     <row r="3" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="23" t="s">
-        <v>320</v>
+        <v>339</v>
       </c>
       <c r="B3" s="23" t="s">
-        <v>321</v>
+        <v>340</v>
       </c>
       <c r="C3" s="24" t="s">
-        <v>322</v>
+        <v>341</v>
       </c>
       <c r="D3" s="25" t="s">
-        <v>323</v>
+        <v>342</v>
       </c>
       <c r="E3" s="25" t="s">
-        <v>324</v>
+        <v>343</v>
       </c>
     </row>
     <row r="4" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="26" t="s">
-        <v>325</v>
+        <v>344</v>
       </c>
       <c r="B4" s="26" t="s">
-        <v>326</v>
+        <v>345</v>
       </c>
       <c r="C4" s="27" t="s">
-        <v>327</v>
+        <v>346</v>
       </c>
       <c r="D4" s="28" t="s">
-        <v>328</v>
+        <v>347</v>
       </c>
       <c r="E4" s="28" t="s">
-        <v>329</v>
+        <v>348</v>
       </c>
     </row>
     <row r="5" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="23" t="s">
-        <v>330</v>
+        <v>349</v>
       </c>
       <c r="B5" s="23" t="s">
-        <v>331</v>
+        <v>350</v>
       </c>
       <c r="C5" s="24" t="s">
-        <v>332</v>
+        <v>351</v>
       </c>
       <c r="D5" s="25" t="s">
-        <v>333</v>
+        <v>352</v>
       </c>
       <c r="E5" s="25" t="s">
-        <v>334</v>
+        <v>353</v>
       </c>
     </row>
     <row r="6" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="26" t="s">
-        <v>335</v>
+        <v>354</v>
       </c>
       <c r="B6" s="26" t="s">
-        <v>336</v>
+        <v>355</v>
       </c>
       <c r="C6" s="27" t="s">
-        <v>337</v>
+        <v>356</v>
       </c>
       <c r="D6" s="28" t="s">
-        <v>338</v>
+        <v>357</v>
       </c>
       <c r="E6" s="28" t="s">
-        <v>339</v>
+        <v>358</v>
       </c>
     </row>
     <row r="7" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="23" t="s">
-        <v>340</v>
+        <v>359</v>
       </c>
       <c r="B7" s="23" t="s">
-        <v>341</v>
+        <v>360</v>
       </c>
       <c r="C7" s="24" t="s">
-        <v>342</v>
+        <v>361</v>
       </c>
       <c r="D7" s="25" t="s">
-        <v>343</v>
+        <v>362</v>
       </c>
       <c r="E7" s="25" t="s">
-        <v>344</v>
+        <v>363</v>
       </c>
     </row>
   </sheetData>
@@ -3357,86 +3494,86 @@
   <sheetData>
     <row r="1" ht="36" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="41" t="s">
-        <v>345</v>
+        <v>364</v>
       </c>
       <c r="B1" s="41"/>
       <c r="C1" s="41"/>
     </row>
     <row r="2" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="42" t="s">
-        <v>346</v>
+        <v>365</v>
       </c>
       <c r="B2" s="42" t="s">
-        <v>347</v>
+        <v>366</v>
       </c>
       <c r="C2" s="42" t="s">
-        <v>348</v>
+        <v>367</v>
       </c>
     </row>
     <row r="3" ht="42" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="15" t="s">
-        <v>349</v>
+        <v>368</v>
       </c>
       <c r="B3" s="16" t="s">
-        <v>350</v>
+        <v>369</v>
       </c>
       <c r="C3" s="17" t="s">
-        <v>351</v>
+        <v>370</v>
       </c>
     </row>
     <row r="4" ht="42" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="18" t="s">
-        <v>352</v>
+        <v>371</v>
       </c>
       <c r="B4" s="19" t="s">
-        <v>353</v>
+        <v>372</v>
       </c>
       <c r="C4" s="20" t="s">
-        <v>354</v>
+        <v>373</v>
       </c>
     </row>
     <row r="5" ht="42" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="15" t="s">
-        <v>355</v>
+        <v>374</v>
       </c>
       <c r="B5" s="16" t="s">
-        <v>356</v>
+        <v>375</v>
       </c>
       <c r="C5" s="17" t="s">
-        <v>357</v>
+        <v>376</v>
       </c>
     </row>
     <row r="6" ht="42" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="18" t="s">
-        <v>358</v>
+        <v>377</v>
       </c>
       <c r="B6" s="19" t="s">
-        <v>359</v>
+        <v>378</v>
       </c>
       <c r="C6" s="20" t="s">
-        <v>360</v>
+        <v>379</v>
       </c>
     </row>
     <row r="7" ht="42" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="15" t="s">
-        <v>361</v>
+        <v>380</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>362</v>
+        <v>381</v>
       </c>
       <c r="C7" s="17" t="s">
-        <v>363</v>
+        <v>382</v>
       </c>
     </row>
     <row r="8" ht="42" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="18" t="s">
-        <v>364</v>
+        <v>383</v>
       </c>
       <c r="B8" s="19" t="s">
-        <v>365</v>
+        <v>384</v>
       </c>
       <c r="C8" s="20" t="s">
-        <v>366</v>
+        <v>385</v>
       </c>
     </row>
   </sheetData>

</xml_diff>